<commit_message>
feat: actualizados archivos en data
</commit_message>
<xml_diff>
--- a/data/entrenamiento_modelo.xlsx
+++ b/data/entrenamiento_modelo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="34">
   <si>
     <t>Jugador / Favorito</t>
   </si>
@@ -25,88 +25,94 @@
     <t>Circuito</t>
   </si>
   <si>
-    <t>Marco Cecchinato</t>
+    <t>Mayar Sherif</t>
   </si>
   <si>
     <t>SI</t>
   </si>
   <si>
+    <t>WTA</t>
+  </si>
+  <si>
+    <t>Alvaro Guillen Meza</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
     <t>Challenger M</t>
   </si>
   <si>
-    <t>Luisina Giovannini</t>
-  </si>
-  <si>
-    <t>WTA</t>
-  </si>
-  <si>
-    <t>Mia Ristic</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>Michele Ribecai</t>
-  </si>
-  <si>
-    <t>Oriol Roca Batalla</t>
-  </si>
-  <si>
-    <t>Daniel Jade</t>
-  </si>
-  <si>
-    <t>Luca Van Assche</t>
+    <t>Benjamin Hassan</t>
+  </si>
+  <si>
+    <t>Matteo Martineau</t>
+  </si>
+  <si>
+    <t>Hernan Casanova</t>
+  </si>
+  <si>
+    <t>Sebastian Ofner</t>
+  </si>
+  <si>
+    <t>Nicolas Barrientos</t>
+  </si>
+  <si>
+    <t>Duje Ajdukovic</t>
+  </si>
+  <si>
+    <t>Valentin Basel</t>
+  </si>
+  <si>
+    <t>Juan Bautista Otegui</t>
+  </si>
+  <si>
+    <t>Imanol Lopez Morillo</t>
+  </si>
+  <si>
+    <t>Sumit Nagal</t>
+  </si>
+  <si>
+    <t>Radu David Turcanu</t>
+  </si>
+  <si>
+    <t>Denis Yevseyev</t>
+  </si>
+  <si>
+    <t>Sascha Gueymard Wayenburg</t>
+  </si>
+  <si>
+    <t>Martin Krumich</t>
+  </si>
+  <si>
+    <t>Sandro Kopp</t>
   </si>
   <si>
     <t>Facundo Diaz Acosta</t>
   </si>
   <si>
-    <t>Stefano Travaglia</t>
-  </si>
-  <si>
-    <t>Maks Kasnikowski</t>
-  </si>
-  <si>
-    <t>Jazmin Ortenzi</t>
-  </si>
-  <si>
-    <t>Roberto Carballes Baena</t>
-  </si>
-  <si>
-    <t>Joao Lucas Reis Da Silva</t>
-  </si>
-  <si>
-    <t>Gonzalo Villanueva</t>
-  </si>
-  <si>
-    <t>Hernan Casanova</t>
-  </si>
-  <si>
-    <t>Cosme Rolland De Ravel</t>
-  </si>
-  <si>
-    <t>Chun-Hsin Tseng</t>
-  </si>
-  <si>
-    <t>Gustavo Heide</t>
+    <t>Pyotr Nesterov</t>
+  </si>
+  <si>
+    <t>Tommaso Compagnucci</t>
+  </si>
+  <si>
+    <t>Manas Dhamne</t>
+  </si>
+  <si>
+    <t>Marko Topo</t>
+  </si>
+  <si>
+    <t>Philip Henning</t>
+  </si>
+  <si>
+    <t>Francesco Passaro</t>
+  </si>
+  <si>
+    <t>Max Alcala Gurri</t>
   </si>
   <si>
     <t>Nick Hardt</t>
-  </si>
-  <si>
-    <t>Luciano Emanuel Ambrogi</t>
-  </si>
-  <si>
-    <t>Daniel Rincon</t>
-  </si>
-  <si>
-    <t>Anastasiia Sobolieva</t>
-  </si>
-  <si>
-    <t>Dalibor Svrcina</t>
-  </si>
-  <si>
-    <t>Kilian Feldbausch</t>
   </si>
 </sst>
 </file>
@@ -133,7 +139,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -150,12 +156,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCFE2F3"/>
-        <bgColor rgb="FFCFE2F3"/>
       </patternFill>
     </fill>
   </fills>
@@ -179,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -195,10 +195,7 @@
     <xf borderId="1" fillId="3" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -420,7 +417,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="25.5"/>
     <col customWidth="1" min="2" max="2" width="14.13"/>
-    <col customWidth="1" min="4" max="4" width="13.5"/>
+    <col customWidth="1" min="4" max="4" width="18.63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -442,12 +439,12 @@
         <v>4</v>
       </c>
       <c r="B2" s="4">
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -456,27 +453,27 @@
         <v>7</v>
       </c>
       <c r="B3" s="4">
-        <v>0.68</v>
+        <v>0.62</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="6" t="s">
         <v>8</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" s="4">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -489,8 +486,8 @@
       <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>6</v>
+      <c r="D5" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -498,13 +495,13 @@
         <v>12</v>
       </c>
       <c r="B6" s="4">
-        <v>0.58</v>
+        <v>0.72</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -512,13 +509,13 @@
         <v>13</v>
       </c>
       <c r="B7" s="4">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -526,13 +523,13 @@
         <v>14</v>
       </c>
       <c r="B8" s="4">
-        <v>0.54</v>
+        <v>0.62</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>6</v>
+      <c r="D8" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -540,268 +537,374 @@
         <v>15</v>
       </c>
       <c r="B9" s="4">
-        <v>0.54</v>
+        <v>0.63</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>6</v>
+      <c r="D9" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" s="4">
-        <v>0.53</v>
+        <v>0.66</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B11" s="4">
-        <v>0.52</v>
+        <v>0.62</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B12" s="4">
-        <v>0.76</v>
+        <v>0.66</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="6" t="s">
         <v>8</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="4">
-        <v>0.64</v>
+        <v>0.67</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="4">
-        <v>0.61</v>
+        <v>0.71</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="4">
-        <v>0.72</v>
+        <v>0.58</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>6</v>
+      <c r="D15" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="4">
-        <v>0.71</v>
+        <v>0.61</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B17" s="4">
         <v>0.68</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B18" s="4">
-        <v>0.53</v>
+        <v>0.78</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="4">
-        <v>0.58</v>
+        <v>0.56</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>6</v>
+      <c r="D19" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="4">
-        <v>0.63</v>
+        <v>0.68</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>6</v>
+      <c r="D20" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="4">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B22" s="4">
-        <v>0.73</v>
+        <v>0.64</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>6</v>
+      <c r="D22" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B23" s="4">
-        <v>0.64</v>
+        <v>0.57</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B24" s="4">
-        <v>0.62</v>
+        <v>0.71</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D24" s="6" t="s">
-        <v>8</v>
+      <c r="D24" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B25" s="4">
-        <v>0.54</v>
+        <v>0.64</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B26" s="4">
-        <v>0.58</v>
+        <v>0.68</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4">
+        <v>0.62</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4">
+        <v>0.64</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4">
+        <v>0.85</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B30" s="4">
+        <v>0.82</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B31" s="4">
         <v>0.61</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>6</v>
+      <c r="C31" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" s="4">
+        <v>0.64</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" s="4">
+        <v>0.57</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B34" s="4">
+        <v>0.65</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D34">
+      <formula1>"ATP,WTA,Challenger M,Challenger F"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C34">
+      <formula1>"NO,SI"</formula1>
+    </dataValidation>
+  </dataValidations>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>